<commit_message>
📊 업데이트 - 2026-09-14 16:07
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA34"/>
+  <dimension ref="A1:AA28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,41 +556,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>03:45</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Aveley FC</t>
+          <t>FC Porto B</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wingate &amp; Finchley</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+          <t>Vizela</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="E2" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.9</v>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>45</v>
-      </c>
+          <t>원정승</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
-        <v>434</v>
+        <v>26</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>IL</t>
+          <t>Portugal Segunda Liga +</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -598,23 +602,17 @@
           <t>원정정배</t>
         </is>
       </c>
-      <c r="M2" t="n">
-        <v>45</v>
-      </c>
-      <c r="N2" t="n">
-        <v>29</v>
-      </c>
-      <c r="O2" t="n">
-        <v>25</v>
-      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -622,58 +620,52 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S2" t="n">
-        <v>76.2</v>
-      </c>
-      <c r="T2" t="n">
-        <v>59.7</v>
-      </c>
-      <c r="U2" t="n">
-        <v>56.7</v>
-      </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="n">
-        <v>49.1</v>
+        <v>19.2</v>
       </c>
       <c r="W2" t="n">
-        <v>24</v>
+        <v>15.4</v>
       </c>
       <c r="X2" t="n">
-        <v>27</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="Y2" t="n">
-        <v>55.5</v>
+        <v>69.2</v>
       </c>
       <c r="Z2" t="n">
-        <v>32</v>
+        <v>38.5</v>
       </c>
       <c r="AA2" t="n">
-        <v>434</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Shabab Al Ahli Dubai</t>
+          <t>Sporting CP B</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Tractor Sazi</t>
+          <t>Lusitânia Lourosa</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.6</v>
+        <v>2.1</v>
       </c>
       <c r="E3" t="n">
-        <v>3.8</v>
+        <v>2.9</v>
       </c>
       <c r="F3" t="n">
-        <v>5.2</v>
+        <v>3.7</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -682,11 +674,11 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>296</v>
+        <v>26</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>World AFC Champions League Elite +</t>
+          <t>Portugal Segunda Liga +</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -721,68 +713,66 @@
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="n">
-        <v>45.9</v>
+        <v>46.2</v>
       </c>
       <c r="W3" t="n">
-        <v>21.3</v>
+        <v>42.3</v>
       </c>
       <c r="X3" t="n">
-        <v>32.8</v>
+        <v>11.5</v>
       </c>
       <c r="Y3" t="n">
-        <v>61.8</v>
+        <v>30.8</v>
       </c>
       <c r="Z3" t="n">
-        <v>40.9</v>
+        <v>15.4</v>
       </c>
       <c r="AA3" t="n">
-        <v>296</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Neftchi Fergana</t>
+          <t>KAMAZ</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Quwa Al Jawiya</t>
+          <t>Chelyabinsk</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1.5</v>
+        <v>2.3</v>
       </c>
       <c r="E4" t="n">
-        <v>3.9</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
-        <v>6.2</v>
+        <v>3.1</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>원정승</t>
         </is>
       </c>
-      <c r="H4" t="n">
-        <v>37</v>
-      </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>127</v>
+        <v>94</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>World AFC Champions League Elite +</t>
+          <t>Russia First League +</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -790,23 +780,17 @@
           <t>홈정배</t>
         </is>
       </c>
-      <c r="M4" t="n">
-        <v>31</v>
-      </c>
-      <c r="N4" t="n">
-        <v>32</v>
-      </c>
-      <c r="O4" t="n">
-        <v>37</v>
-      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -814,81 +798,75 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S4" t="n">
-        <v>57.7</v>
-      </c>
-      <c r="T4" t="n">
-        <v>56.3</v>
-      </c>
-      <c r="U4" t="n">
-        <v>35.3</v>
-      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
       <c r="V4" t="n">
-        <v>44.1</v>
+        <v>30.9</v>
       </c>
       <c r="W4" t="n">
-        <v>20.5</v>
+        <v>23.4</v>
       </c>
       <c r="X4" t="n">
-        <v>35.4</v>
+        <v>45.7</v>
       </c>
       <c r="Y4" t="n">
-        <v>59.1</v>
+        <v>50</v>
       </c>
       <c r="Z4" t="n">
-        <v>38.6</v>
+        <v>23.4</v>
       </c>
       <c r="AA4" t="n">
-        <v>127</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Banfield</t>
+          <t>Veles</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Barracas Central</t>
+          <t>FC Sochi</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2.4</v>
+        <v>3.7</v>
       </c>
       <c r="E5" t="n">
-        <v>2.9</v>
+        <v>3.3</v>
       </c>
       <c r="F5" t="n">
-        <v>3.3</v>
+        <v>2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>311</v>
+        <v>39</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Argentina Liga Profesional +</t>
+          <t>Russia First League +</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>★</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -913,22 +891,22 @@
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="n">
-        <v>42.1</v>
+        <v>25.6</v>
       </c>
       <c r="W5" t="n">
-        <v>21.9</v>
+        <v>28.2</v>
       </c>
       <c r="X5" t="n">
-        <v>36</v>
+        <v>46.2</v>
       </c>
       <c r="Y5" t="n">
-        <v>59.8</v>
+        <v>56.4</v>
       </c>
       <c r="Z5" t="n">
-        <v>39.9</v>
+        <v>28.2</v>
       </c>
       <c r="AA5" t="n">
-        <v>311</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
@@ -939,31 +917,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Deportivo Riestra</t>
+          <t>Banfield</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Lanus</t>
+          <t>Barracas Central</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>3.1</v>
+        <v>2.4</v>
       </c>
       <c r="E6" t="n">
-        <v>2.7</v>
+        <v>2.9</v>
       </c>
       <c r="F6" t="n">
-        <v>2.6</v>
+        <v>3.3</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>281</v>
+        <v>42</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -977,7 +955,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -1002,48 +980,48 @@
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="n">
-        <v>43.8</v>
+        <v>31</v>
       </c>
       <c r="W6" t="n">
-        <v>21.4</v>
+        <v>26.2</v>
       </c>
       <c r="X6" t="n">
-        <v>34.9</v>
+        <v>42.9</v>
       </c>
       <c r="Y6" t="n">
-        <v>61.9</v>
+        <v>40.5</v>
       </c>
       <c r="Z6" t="n">
-        <v>41.3</v>
+        <v>26.2</v>
       </c>
       <c r="AA6" t="n">
-        <v>281</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bahia</t>
+          <t>Deportivo Riestra</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Remo</t>
+          <t>Lanus</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.4</v>
+        <v>3.1</v>
       </c>
       <c r="E7" t="n">
-        <v>4.5</v>
+        <v>2.7</v>
       </c>
       <c r="F7" t="n">
-        <v>6.8</v>
+        <v>2.6</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1052,11 +1030,11 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>270</v>
+        <v>12</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Brazil Serie A +</t>
+          <t>Argentina Liga Profesional +</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1066,7 +1044,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M7" t="inlineStr"/>
@@ -1091,22 +1069,22 @@
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="n">
-        <v>44.4</v>
+        <v>41.7</v>
       </c>
       <c r="W7" t="n">
-        <v>20.7</v>
+        <v>25</v>
       </c>
       <c r="X7" t="n">
-        <v>34.8</v>
+        <v>33.3</v>
       </c>
       <c r="Y7" t="n">
-        <v>63</v>
+        <v>33.3</v>
       </c>
       <c r="Z7" t="n">
-        <v>41.9</v>
+        <v>16.7</v>
       </c>
       <c r="AA7" t="n">
-        <v>270</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -1136,12 +1114,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>406</v>
+        <v>131</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -1180,22 +1158,22 @@
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="n">
-        <v>40.6</v>
+        <v>34.4</v>
       </c>
       <c r="W8" t="n">
-        <v>22.2</v>
+        <v>22.1</v>
       </c>
       <c r="X8" t="n">
-        <v>37.2</v>
+        <v>43.5</v>
       </c>
       <c r="Y8" t="n">
-        <v>59.1</v>
+        <v>51.9</v>
       </c>
       <c r="Z8" t="n">
-        <v>35.5</v>
+        <v>22.1</v>
       </c>
       <c r="AA8" t="n">
-        <v>406</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9">
@@ -1225,12 +1203,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>305</v>
+        <v>35</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -1269,22 +1247,22 @@
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="n">
-        <v>42.6</v>
+        <v>31.4</v>
       </c>
       <c r="W9" t="n">
-        <v>22</v>
+        <v>28.6</v>
       </c>
       <c r="X9" t="n">
-        <v>35.4</v>
+        <v>40</v>
       </c>
       <c r="Y9" t="n">
-        <v>60.3</v>
+        <v>40</v>
       </c>
       <c r="Z9" t="n">
-        <v>39.7</v>
+        <v>20</v>
       </c>
       <c r="AA9" t="n">
-        <v>305</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10">
@@ -1314,12 +1292,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>444</v>
+        <v>168</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1358,22 +1336,22 @@
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="n">
-        <v>39.9</v>
+        <v>32.1</v>
       </c>
       <c r="W10" t="n">
-        <v>25.2</v>
+        <v>32.1</v>
       </c>
       <c r="X10" t="n">
-        <v>34.9</v>
+        <v>35.7</v>
       </c>
       <c r="Y10" t="n">
-        <v>58.1</v>
+        <v>50.6</v>
       </c>
       <c r="Z10" t="n">
-        <v>36</v>
+        <v>27.4</v>
       </c>
       <c r="AA10" t="n">
-        <v>444</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11">
@@ -1408,7 +1386,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>361</v>
+        <v>93</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -1447,61 +1425,61 @@
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>43.2</v>
+        <v>40.9</v>
       </c>
       <c r="W11" t="n">
-        <v>21.3</v>
+        <v>22.6</v>
       </c>
       <c r="X11" t="n">
-        <v>35.5</v>
+        <v>36.6</v>
       </c>
       <c r="Y11" t="n">
-        <v>62.6</v>
+        <v>61.3</v>
       </c>
       <c r="Z11" t="n">
-        <v>39.1</v>
+        <v>30.1</v>
       </c>
       <c r="AA11" t="n">
-        <v>361</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:45</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Blackburn Rovers U21</t>
+          <t>RED Star FC 93</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Reading U21</t>
+          <t>Metz</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2.9</v>
+        <v>2.4</v>
       </c>
       <c r="E12" t="n">
-        <v>3.9</v>
+        <v>3.2</v>
       </c>
       <c r="F12" t="n">
-        <v>1.9</v>
+        <v>3</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>284</v>
+        <v>165</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>England Premier League 2 Division One +</t>
+          <t>France Ligue 2 +</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1511,7 +1489,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1536,22 +1514,22 @@
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="n">
-        <v>42.3</v>
+        <v>33.3</v>
       </c>
       <c r="W12" t="n">
-        <v>21.1</v>
+        <v>30.9</v>
       </c>
       <c r="X12" t="n">
-        <v>36.6</v>
+        <v>35.8</v>
       </c>
       <c r="Y12" t="n">
-        <v>63</v>
+        <v>49.1</v>
       </c>
       <c r="Z12" t="n">
-        <v>41.5</v>
+        <v>24.2</v>
       </c>
       <c r="AA12" t="n">
-        <v>284</v>
+        <v>165</v>
       </c>
     </row>
     <row r="13">
@@ -1562,22 +1540,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Nottingham Forest U21</t>
+          <t>Jong Utrecht</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Burnley U21</t>
+          <t>Jong Ajax</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1.5</v>
+        <v>2.2</v>
       </c>
       <c r="E13" t="n">
-        <v>4.4</v>
+        <v>3.9</v>
       </c>
       <c r="F13" t="n">
-        <v>4.5</v>
+        <v>2.8</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1586,11 +1564,11 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>287</v>
+        <v>32</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>England Premier League 2 Division One +</t>
+          <t>Netherlands Eerste Divisie +</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1625,61 +1603,61 @@
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="n">
-        <v>43.6</v>
+        <v>43.8</v>
       </c>
       <c r="W13" t="n">
-        <v>21.6</v>
+        <v>15.6</v>
       </c>
       <c r="X13" t="n">
-        <v>34.8</v>
+        <v>40.6</v>
       </c>
       <c r="Y13" t="n">
-        <v>62</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="Z13" t="n">
-        <v>41.1</v>
+        <v>31.2</v>
       </c>
       <c r="AA13" t="n">
-        <v>287</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>West Ham United U21</t>
+          <t>Moreirense</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Liverpool U21</t>
+          <t>Maritimo</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2.3</v>
+        <v>2.5</v>
       </c>
       <c r="E14" t="n">
-        <v>3.8</v>
+        <v>3.1</v>
       </c>
       <c r="F14" t="n">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>293</v>
+        <v>141</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>England Premier League 2 Division One +</t>
+          <t>Portugal Primeira Liga +</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1714,48 +1692,48 @@
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="n">
-        <v>44.7</v>
+        <v>33.3</v>
       </c>
       <c r="W14" t="n">
-        <v>19.8</v>
+        <v>29.1</v>
       </c>
       <c r="X14" t="n">
-        <v>35.5</v>
+        <v>37.6</v>
       </c>
       <c r="Y14" t="n">
-        <v>64.8</v>
+        <v>51.1</v>
       </c>
       <c r="Z14" t="n">
-        <v>42.7</v>
+        <v>23.4</v>
       </c>
       <c r="AA14" t="n">
-        <v>293</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>RED Star FC 93</t>
+          <t>Rio Ave</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Metz</t>
+          <t>Estrela</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="E15" t="n">
         <v>3.2</v>
       </c>
       <c r="F15" t="n">
-        <v>3</v>
+        <v>2.6</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1764,11 +1742,11 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>437</v>
+        <v>153</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>France Ligue 2 +</t>
+          <t>Portugal Primeira Liga +</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1778,7 +1756,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1803,48 +1781,48 @@
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="n">
-        <v>40</v>
+        <v>34.6</v>
       </c>
       <c r="W15" t="n">
-        <v>24.9</v>
+        <v>32.7</v>
       </c>
       <c r="X15" t="n">
-        <v>35</v>
+        <v>32.7</v>
       </c>
       <c r="Y15" t="n">
-        <v>57.9</v>
+        <v>47.1</v>
       </c>
       <c r="Z15" t="n">
-        <v>35.2</v>
+        <v>26.1</v>
       </c>
       <c r="AA15" t="n">
-        <v>437</v>
+        <v>153</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Spartak Kostroma</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>FK Neftekhimik</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1.2</v>
+        <v>1.7</v>
       </c>
       <c r="E16" t="n">
-        <v>6.4</v>
+        <v>3.6</v>
       </c>
       <c r="F16" t="n">
-        <v>15.5</v>
+        <v>4.8</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1853,11 +1831,11 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>268</v>
+        <v>37</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Italy Serie A +</t>
+          <t>Russia First League +</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1892,61 +1870,61 @@
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
       <c r="V16" t="n">
-        <v>44</v>
+        <v>43.2</v>
       </c>
       <c r="W16" t="n">
-        <v>20.9</v>
+        <v>35.1</v>
       </c>
       <c r="X16" t="n">
-        <v>35.1</v>
+        <v>21.6</v>
       </c>
       <c r="Y16" t="n">
-        <v>63.1</v>
+        <v>43.2</v>
       </c>
       <c r="Z16" t="n">
-        <v>42.2</v>
+        <v>24.3</v>
       </c>
       <c r="AA16" t="n">
-        <v>268</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Shinnik Yaroslavl</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AS Roma</t>
+          <t>Ural</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>6.1</v>
+        <v>3.4</v>
       </c>
       <c r="E17" t="n">
-        <v>4.2</v>
+        <v>3.2</v>
       </c>
       <c r="F17" t="n">
-        <v>1.6</v>
+        <v>2.1</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>270</v>
+        <v>66</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Italy Serie A +</t>
+          <t>Russia First League +</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1981,48 +1959,48 @@
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="n">
-        <v>43.7</v>
+        <v>34.8</v>
       </c>
       <c r="W17" t="n">
-        <v>20.7</v>
+        <v>27.3</v>
       </c>
       <c r="X17" t="n">
-        <v>35.6</v>
+        <v>37.9</v>
       </c>
       <c r="Y17" t="n">
-        <v>63.3</v>
+        <v>51.5</v>
       </c>
       <c r="Z17" t="n">
-        <v>42.6</v>
+        <v>27.3</v>
       </c>
       <c r="AA17" t="n">
-        <v>270</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Jong PSV U21</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Jong AZ</t>
+          <t>Real Betis</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2.6</v>
+        <v>1.9</v>
       </c>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="F18" t="n">
-        <v>2.3</v>
+        <v>3.8</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -2031,11 +2009,11 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>282</v>
+        <v>41</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Netherlands Eerste Divisie +</t>
+          <t>Spain La Liga +</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -2045,7 +2023,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M18" t="inlineStr"/>
@@ -2070,61 +2048,61 @@
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="n">
-        <v>43.6</v>
+        <v>43.9</v>
       </c>
       <c r="W18" t="n">
-        <v>21.3</v>
+        <v>22</v>
       </c>
       <c r="X18" t="n">
-        <v>35.1</v>
+        <v>34.1</v>
       </c>
       <c r="Y18" t="n">
-        <v>63.5</v>
+        <v>63.4</v>
       </c>
       <c r="Z18" t="n">
-        <v>42.9</v>
+        <v>41.5</v>
       </c>
       <c r="AA18" t="n">
-        <v>282</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Jong Utrecht</t>
+          <t>Celta de Vigo II</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Jong Ajax</t>
+          <t>Eibar</t>
         </is>
       </c>
       <c r="D19" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E19" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F19" t="n">
         <v>2.2</v>
       </c>
-      <c r="E19" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="F19" t="n">
-        <v>2.8</v>
-      </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
-        <v>303</v>
+        <v>38</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Netherlands Eerste Divisie +</t>
+          <t>Spain Segunda División +</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2134,7 +2112,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -2159,61 +2137,61 @@
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>44.2</v>
+        <v>31.6</v>
       </c>
       <c r="W19" t="n">
-        <v>20.1</v>
+        <v>31.6</v>
       </c>
       <c r="X19" t="n">
-        <v>35.6</v>
+        <v>36.8</v>
       </c>
       <c r="Y19" t="n">
-        <v>63.4</v>
+        <v>50</v>
       </c>
       <c r="Z19" t="n">
-        <v>40.9</v>
+        <v>26.3</v>
       </c>
       <c r="AA19" t="n">
-        <v>303</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SC Braga</t>
+          <t>Atletico Torque</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Estoril</t>
+          <t>Liverpool Montevideo</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1.4</v>
+        <v>3.3</v>
       </c>
       <c r="E20" t="n">
-        <v>4.5</v>
+        <v>3.2</v>
       </c>
       <c r="F20" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>홈승</t>
+          <t>원정승</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
-        <v>270</v>
+        <v>64</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Portugal Primeira Liga +</t>
+          <t>Uruguay Primera División +</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2223,7 +2201,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -2248,66 +2226,64 @@
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="n">
-        <v>44.1</v>
+        <v>29.7</v>
       </c>
       <c r="W20" t="n">
-        <v>21.1</v>
+        <v>29.7</v>
       </c>
       <c r="X20" t="n">
-        <v>34.8</v>
+        <v>40.6</v>
       </c>
       <c r="Y20" t="n">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="Z20" t="n">
-        <v>41.9</v>
+        <v>28.1</v>
       </c>
       <c r="AA20" t="n">
-        <v>270</v>
+        <v>64</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Moreirense</t>
+          <t>Bahia</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Maritimo</t>
+          <t>Remo</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2.5</v>
+        <v>1.4</v>
       </c>
       <c r="E21" t="n">
-        <v>3.1</v>
+        <v>4.5</v>
       </c>
       <c r="F21" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
+        <v>6.8</v>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
       <c r="I21" t="n">
-        <v>415</v>
+        <v>2</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Portugal Primeira Liga +</t>
+          <t>Brazil Serie A +</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>❓</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2337,71 +2313,69 @@
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>40.2</v>
+        <v>100</v>
       </c>
       <c r="W21" t="n">
-        <v>24.1</v>
+        <v>0</v>
       </c>
       <c r="X21" t="n">
-        <v>35.7</v>
+        <v>0</v>
       </c>
       <c r="Y21" t="n">
-        <v>58.8</v>
+        <v>50</v>
       </c>
       <c r="Z21" t="n">
-        <v>35.4</v>
+        <v>0</v>
       </c>
       <c r="AA21" t="n">
-        <v>415</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Rio Ave</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Estrela</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>2.6</v>
+        <v>1.2</v>
       </c>
       <c r="E22" t="n">
-        <v>3.2</v>
+        <v>6.4</v>
       </c>
       <c r="F22" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
+        <v>15.5</v>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
       <c r="I22" t="n">
-        <v>429</v>
+        <v>0</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Portugal Primeira Liga +</t>
+          <t>Italy Serie A +</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>❓</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
@@ -2425,72 +2399,60 @@
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
-      <c r="V22" t="n">
-        <v>40.6</v>
-      </c>
-      <c r="W22" t="n">
-        <v>24.9</v>
-      </c>
-      <c r="X22" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>56.9</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>35.9</v>
-      </c>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="n">
-        <v>429</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>18:45</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>FC Porto B</t>
+          <t>Inter</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Vizela</t>
+          <t>Udinese</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>3.8</v>
+        <v>1.3</v>
       </c>
       <c r="E23" t="n">
-        <v>3.3</v>
+        <v>6.3</v>
       </c>
       <c r="F23" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
+        <v>12.5</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
       <c r="I23" t="n">
-        <v>296</v>
+        <v>1</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Portugal Segunda Liga +</t>
+          <t>Italy Serie A +</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>❓</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M23" t="inlineStr"/>
@@ -2515,71 +2477,69 @@
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
       <c r="V23" t="n">
-        <v>41.6</v>
+        <v>0</v>
       </c>
       <c r="W23" t="n">
-        <v>20.3</v>
+        <v>100</v>
       </c>
       <c r="X23" t="n">
-        <v>38.2</v>
+        <v>0</v>
       </c>
       <c r="Y23" t="n">
-        <v>63.2</v>
+        <v>100</v>
       </c>
       <c r="Z23" t="n">
-        <v>41.6</v>
+        <v>100</v>
       </c>
       <c r="AA23" t="n">
-        <v>296</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Sporting CP B</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Lusitânia Lourosa</t>
+          <t>AS Roma</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>2.1</v>
+        <v>6.1</v>
       </c>
       <c r="E24" t="n">
-        <v>2.9</v>
+        <v>4.2</v>
       </c>
       <c r="F24" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr"/>
+        <v>1.6</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
       <c r="I24" t="n">
-        <v>296</v>
+        <v>2</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Portugal Segunda Liga +</t>
+          <t>Italy Serie A +</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>❓</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M24" t="inlineStr"/>
@@ -2604,71 +2564,69 @@
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="n">
-        <v>43.9</v>
+        <v>0</v>
       </c>
       <c r="W24" t="n">
-        <v>23.3</v>
+        <v>0</v>
       </c>
       <c r="X24" t="n">
-        <v>32.8</v>
+        <v>100</v>
       </c>
       <c r="Y24" t="n">
-        <v>59.8</v>
+        <v>100</v>
       </c>
       <c r="Z24" t="n">
-        <v>39.5</v>
+        <v>100</v>
       </c>
       <c r="AA24" t="n">
-        <v>296</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>KAMAZ</t>
+          <t>Jong PSV U21</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Chelyabinsk</t>
+          <t>Jong AZ</t>
         </is>
       </c>
       <c r="D25" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E25" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" t="n">
         <v>2.3</v>
       </c>
-      <c r="E25" t="n">
-        <v>3</v>
-      </c>
-      <c r="F25" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
       <c r="I25" t="n">
-        <v>368</v>
+        <v>9</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Russia First League +</t>
+          <t>Netherlands Eerste Divisie +</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>❓</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -2693,66 +2651,64 @@
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
       <c r="V25" t="n">
-        <v>40.5</v>
+        <v>22.2</v>
       </c>
       <c r="W25" t="n">
-        <v>22.3</v>
+        <v>33.3</v>
       </c>
       <c r="X25" t="n">
-        <v>37.2</v>
+        <v>44.4</v>
       </c>
       <c r="Y25" t="n">
-        <v>59.5</v>
+        <v>55.6</v>
       </c>
       <c r="Z25" t="n">
-        <v>37.2</v>
+        <v>44.4</v>
       </c>
       <c r="AA25" t="n">
-        <v>368</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Spartak Kostroma</t>
+          <t>Bodo/Glimt</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>FK Neftekhimik</t>
+          <t>Sandefjord</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
       <c r="E26" t="n">
-        <v>3.6</v>
+        <v>8.5</v>
       </c>
       <c r="F26" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr"/>
+        <v>14.5</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
       <c r="I26" t="n">
-        <v>306</v>
+        <v>0</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Russia First League +</t>
+          <t>Norway Eliteserien +</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>❓</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2781,72 +2737,60 @@
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
-      <c r="V26" t="n">
-        <v>43.8</v>
-      </c>
-      <c r="W26" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="X26" t="n">
-        <v>33.7</v>
-      </c>
-      <c r="Y26" t="n">
-        <v>60.5</v>
-      </c>
-      <c r="Z26" t="n">
-        <v>39.9</v>
-      </c>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
       <c r="AA26" t="n">
-        <v>306</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Shinnik Yaroslavl</t>
+          <t>SC Braga</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ural</t>
+          <t>Estoril</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>3.4</v>
+        <v>1.4</v>
       </c>
       <c r="E27" t="n">
-        <v>3.2</v>
+        <v>4.5</v>
       </c>
       <c r="F27" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
       <c r="I27" t="n">
-        <v>335</v>
+        <v>2</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Russia First League +</t>
+          <t>Portugal Primeira Liga +</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>❓</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -2871,66 +2815,64 @@
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="n">
-        <v>42.1</v>
+        <v>50</v>
       </c>
       <c r="W27" t="n">
-        <v>22.4</v>
+        <v>50</v>
       </c>
       <c r="X27" t="n">
-        <v>35.5</v>
+        <v>0</v>
       </c>
       <c r="Y27" t="n">
-        <v>60.6</v>
+        <v>50</v>
       </c>
       <c r="Z27" t="n">
-        <v>39.1</v>
+        <v>0</v>
       </c>
       <c r="AA27" t="n">
-        <v>335</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Veles</t>
+          <t>Gaziantep FK</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>FC Sochi</t>
+          <t>Fenerbahçe</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3.7</v>
+        <v>5.8</v>
       </c>
       <c r="E28" t="n">
-        <v>3.3</v>
+        <v>4.2</v>
       </c>
       <c r="F28" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
         <v>2</v>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="n">
-        <v>308</v>
-      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Russia First League +</t>
+          <t>Turkey Süper Lig +</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>❓</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2960,556 +2902,22 @@
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
       <c r="V28" t="n">
-        <v>41.6</v>
+        <v>0</v>
       </c>
       <c r="W28" t="n">
-        <v>21.8</v>
+        <v>0</v>
       </c>
       <c r="X28" t="n">
-        <v>36.7</v>
+        <v>100</v>
       </c>
       <c r="Y28" t="n">
-        <v>62</v>
+        <v>100</v>
       </c>
       <c r="Z28" t="n">
-        <v>40.3</v>
+        <v>50</v>
       </c>
       <c r="AA28" t="n">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>18:30</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Celta de Vigo II</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Eibar</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="E29" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="F29" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="n">
-        <v>307</v>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>Spain Segunda División +</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr"/>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="W29" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="X29" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="Y29" t="n">
-        <v>61.2</v>
-      </c>
-      <c r="Z29" t="n">
-        <v>40.1</v>
-      </c>
-      <c r="AA29" t="n">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Gaziantep FK</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Fenerbahçe</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="E30" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="F30" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="n">
-        <v>270</v>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Turkey Süper Lig +</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="n">
-        <v>43.7</v>
-      </c>
-      <c r="W30" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="X30" t="n">
-        <v>35.6</v>
-      </c>
-      <c r="Y30" t="n">
-        <v>63.3</v>
-      </c>
-      <c r="Z30" t="n">
-        <v>42.2</v>
-      </c>
-      <c r="AA30" t="n">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>22:00</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Atletico Torque</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Liverpool Montevideo</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="E31" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="F31" t="n">
         <v>2</v>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="n">
-        <v>333</v>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>Uruguay Primera División +</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
-      <c r="U31" t="inlineStr"/>
-      <c r="V31" t="n">
-        <v>41.1</v>
-      </c>
-      <c r="W31" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="X31" t="n">
-        <v>36</v>
-      </c>
-      <c r="Y31" t="n">
-        <v>60.4</v>
-      </c>
-      <c r="Z31" t="n">
-        <v>39.3</v>
-      </c>
-      <c r="AA31" t="n">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Esteghlal FC</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Al Sadd</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="E32" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="F32" t="n">
-        <v>2</v>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="n">
-        <v>326</v>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>World AFC Champions League Elite +</t>
-        </is>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>원정정배</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="n">
-        <v>40.5</v>
-      </c>
-      <c r="W32" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="X32" t="n">
-        <v>35.9</v>
-      </c>
-      <c r="Y32" t="n">
-        <v>61</v>
-      </c>
-      <c r="Z32" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="AA32" t="n">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Al-Ahli Jeddah</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Pakhtakor</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="E33" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="F33" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="n">
-        <v>269</v>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>World AFC Champions League Elite +</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S33" t="inlineStr"/>
-      <c r="T33" t="inlineStr"/>
-      <c r="U33" t="inlineStr"/>
-      <c r="V33" t="n">
-        <v>44.2</v>
-      </c>
-      <c r="W33" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="X33" t="n">
-        <v>34.9</v>
-      </c>
-      <c r="Y33" t="n">
-        <v>63.2</v>
-      </c>
-      <c r="Z33" t="n">
-        <v>42.4</v>
-      </c>
-      <c r="AA33" t="n">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Al-Qadisiyah FC</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Al-Wasl FC</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="E34" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="F34" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="n">
-        <v>271</v>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>World AFC Champions League Elite +</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>⚡</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>홈정배</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S34" t="inlineStr"/>
-      <c r="T34" t="inlineStr"/>
-      <c r="U34" t="inlineStr"/>
-      <c r="V34" t="n">
-        <v>44.6</v>
-      </c>
-      <c r="W34" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="X34" t="n">
-        <v>34.7</v>
-      </c>
-      <c r="Y34" t="n">
-        <v>63.5</v>
-      </c>
-      <c r="Z34" t="n">
-        <v>42.1</v>
-      </c>
-      <c r="AA34" t="n">
-        <v>271</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-15 16:25
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -556,7 +556,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -645,7 +645,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>03:45</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -734,7 +734,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>03:45</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -823,7 +823,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -912,7 +912,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1001,7 +1001,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>03:45</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1090,7 +1090,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1179,7 +1179,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1268,7 +1268,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>03:45</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1357,7 +1357,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>03:45</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1446,7 +1446,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1535,7 +1535,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1624,7 +1624,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>03:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1713,7 +1713,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1800,7 +1800,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>03:00</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1877,7 +1877,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>03:45</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1964,7 +1964,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2041,7 +2041,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">

</xml_diff>

<commit_message>
📊 업데이트 - 2026-09-16 16:43
</commit_message>
<xml_diff>
--- a/today_ai_all_picks.xlsx
+++ b/today_ai_all_picks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA19"/>
+  <dimension ref="A1:AA28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -556,40 +556,42 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MSV Duisburg</t>
+          <t>Bayer Leverkusen</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Havelse</t>
+          <t>Celje</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="E2" t="n">
-        <v>4.8</v>
+        <v>8.6</v>
       </c>
       <c r="F2" t="n">
-        <v>7.5</v>
+        <v>17</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
       <c r="I2" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Germany 3. Liga +</t>
+          <t>World UEFA Europa League</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -621,64 +623,68 @@
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="n">
+        <v>69.8</v>
+      </c>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="n">
-        <v>80</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="W2" t="n">
-        <v>10</v>
+        <v>12.8</v>
       </c>
       <c r="X2" t="n">
-        <v>10</v>
+        <v>12.6</v>
       </c>
       <c r="Y2" t="n">
-        <v>70</v>
+        <v>69.8</v>
       </c>
       <c r="Z2" t="n">
-        <v>20</v>
+        <v>46.9</v>
       </c>
       <c r="AA2" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>03:45</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hibernian</t>
+          <t>Olympiakos Piraeus</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Kilmarnock</t>
+          <t>Jagiellonia</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E3" t="n">
-        <v>4.4</v>
+        <v>4.8</v>
       </c>
       <c r="F3" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
       <c r="I3" t="n">
-        <v>11</v>
+        <v>60</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Scotland Premiership +</t>
+          <t>World UEFA Europa League</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -710,69 +716,73 @@
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
+      <c r="T3" t="n">
+        <v>65.8</v>
+      </c>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="n">
-        <v>72.7</v>
+        <v>64.3</v>
       </c>
       <c r="W3" t="n">
-        <v>9.1</v>
+        <v>20.4</v>
       </c>
       <c r="X3" t="n">
-        <v>18.2</v>
+        <v>15.3</v>
       </c>
       <c r="Y3" t="n">
-        <v>63.6</v>
+        <v>65.8</v>
       </c>
       <c r="Z3" t="n">
         <v>36.4</v>
       </c>
       <c r="AA3" t="n">
-        <v>11</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>03:45</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Middlesbrough</t>
+          <t>Spartak Moscow</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Millwall</t>
+          <t>Fakel</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="E4" t="n">
-        <v>4.3</v>
+        <v>5.2</v>
       </c>
       <c r="F4" t="n">
-        <v>5.3</v>
+        <v>9.4</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
       <c r="I4" t="n">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>England Championship +</t>
+          <t>Russia Premier League</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -799,25 +809,27 @@
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
+      <c r="T4" t="n">
+        <v>51.1</v>
+      </c>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="n">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="W4" t="n">
-        <v>22.2</v>
+        <v>29.3</v>
       </c>
       <c r="X4" t="n">
-        <v>14.8</v>
+        <v>15.7</v>
       </c>
       <c r="Y4" t="n">
-        <v>70.40000000000001</v>
+        <v>51.1</v>
       </c>
       <c r="Z4" t="n">
-        <v>37</v>
+        <v>27.9</v>
       </c>
       <c r="AA4" t="n">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5">
@@ -828,35 +840,37 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SSV Jahn Regensburg</t>
+          <t>Atletico Madrid</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fortuna Düsseldorf</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2.9</v>
+        <v>1.4</v>
       </c>
       <c r="E5" t="n">
-        <v>3.4</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
-        <v>2.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+          <t>홈승</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
       <c r="I5" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Germany 3. Liga +</t>
+          <t>Spain La Liga</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -866,7 +880,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M5" t="inlineStr"/>
@@ -888,69 +902,73 @@
         </is>
       </c>
       <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
+      <c r="T5" t="n">
+        <v>51.9</v>
+      </c>
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="n">
-        <v>22.7</v>
+        <v>38.6</v>
       </c>
       <c r="W5" t="n">
-        <v>21.2</v>
+        <v>25.7</v>
       </c>
       <c r="X5" t="n">
-        <v>56.1</v>
+        <v>35.7</v>
       </c>
       <c r="Y5" t="n">
-        <v>57.6</v>
+        <v>51.9</v>
       </c>
       <c r="Z5" t="n">
-        <v>30.3</v>
+        <v>30.2</v>
       </c>
       <c r="AA5" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Nautico Recife</t>
+          <t>Sunderland</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Operario-PR</t>
+          <t>AZ Alkmaar</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.9</v>
+        <v>1.6</v>
       </c>
       <c r="E6" t="n">
-        <v>3.3</v>
+        <v>4.3</v>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>5.6</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
       <c r="I6" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Brazil Serie B +</t>
+          <t>World UEFA Europa League</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -977,69 +995,73 @@
         </is>
       </c>
       <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
+      <c r="T6" t="n">
+        <v>59.1</v>
+      </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="n">
-        <v>49.2</v>
+        <v>53.8</v>
       </c>
       <c r="W6" t="n">
-        <v>35.4</v>
+        <v>21.6</v>
       </c>
       <c r="X6" t="n">
-        <v>15.4</v>
+        <v>24.6</v>
       </c>
       <c r="Y6" t="n">
-        <v>46.2</v>
+        <v>59.1</v>
       </c>
       <c r="Z6" t="n">
-        <v>26.2</v>
+        <v>29.9</v>
       </c>
       <c r="AA6" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:45</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bristol City</t>
+          <t>Hansa Rostock</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Lincoln</t>
+          <t>Stuttgart II</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.9</v>
+        <v>1.5</v>
       </c>
       <c r="E7" t="n">
-        <v>3.5</v>
+        <v>4.3</v>
       </c>
       <c r="F7" t="n">
-        <v>3.6</v>
+        <v>5</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>홈승</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
       <c r="I7" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>England Championship +</t>
+          <t>Germany 3. Liga</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>★★</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1066,64 +1088,68 @@
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
+      <c r="T7" t="n">
+        <v>60.1</v>
+      </c>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="n">
-        <v>48.9</v>
+        <v>47.7</v>
       </c>
       <c r="W7" t="n">
-        <v>28.9</v>
+        <v>20.7</v>
       </c>
       <c r="X7" t="n">
-        <v>22.2</v>
+        <v>31.6</v>
       </c>
       <c r="Y7" t="n">
-        <v>45.6</v>
+        <v>60.1</v>
       </c>
       <c r="Z7" t="n">
-        <v>22.2</v>
+        <v>27.7</v>
       </c>
       <c r="AA7" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>01:45</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SG Sonnenhof Grossaspach</t>
+          <t>Ararat-Armenia</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Verl</t>
+          <t>Sparta Praha</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2.1</v>
+        <v>5.2</v>
       </c>
       <c r="E8" t="n">
-        <v>3.8</v>
+        <v>4.1</v>
       </c>
       <c r="F8" t="n">
-        <v>2.7</v>
+        <v>1.6</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>원정승</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
       <c r="I8" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Germany 3. Liga +</t>
+          <t>World UEFA Europa League</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1133,7 +1159,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
@@ -1155,74 +1181,74 @@
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
+      <c r="T8" t="n">
+        <v>60</v>
+      </c>
       <c r="U8" t="inlineStr"/>
       <c r="V8" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="W8" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="X8" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>60</v>
+      </c>
+      <c r="Z8" t="n">
         <v>37.8</v>
       </c>
-      <c r="W8" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="X8" t="n">
-        <v>48.6</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>67.59999999999999</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>40.5</v>
-      </c>
       <c r="AA8" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Würzburger Kickers</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Alemannia Aachen</t>
+          <t>Racing Santander</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3.2</v>
+        <v>1.1</v>
       </c>
       <c r="E9" t="n">
-        <v>3.5</v>
+        <v>14.8</v>
       </c>
       <c r="F9" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
+        <v>31</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
       <c r="I9" t="n">
         <v>60</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Germany 3. Liga +</t>
+          <t>Spain La Liga</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⏭</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1244,22 +1270,24 @@
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
+      <c r="T9" t="n">
+        <v>55</v>
+      </c>
       <c r="U9" t="inlineStr"/>
       <c r="V9" t="n">
-        <v>21.7</v>
+        <v>44.8</v>
       </c>
       <c r="W9" t="n">
-        <v>33.3</v>
+        <v>23.3</v>
       </c>
       <c r="X9" t="n">
-        <v>45</v>
+        <v>31.9</v>
       </c>
       <c r="Y9" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="Z9" t="n">
-        <v>33.3</v>
+        <v>33.7</v>
       </c>
       <c r="AA9" t="n">
         <v>60</v>
@@ -1268,50 +1296,48 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:45</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Falkirk</t>
+          <t>Botafogo</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Heart Of Midlothian</t>
+          <t>Gremio</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3.8</v>
+        <v>1.7</v>
       </c>
       <c r="E10" t="n">
         <v>3.7</v>
       </c>
       <c r="F10" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>원정승</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
+        <v>4.6</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
       <c r="I10" t="n">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Scotland Premiership +</t>
+          <t>Brazil Serie A</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⏭</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1333,69 +1359,69 @@
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
+      <c r="T10" t="n">
+        <v>55.4</v>
+      </c>
       <c r="U10" t="inlineStr"/>
       <c r="V10" t="n">
-        <v>14.3</v>
+        <v>46.1</v>
       </c>
       <c r="W10" t="n">
-        <v>31.4</v>
+        <v>25</v>
       </c>
       <c r="X10" t="n">
-        <v>54.3</v>
+        <v>28.9</v>
       </c>
       <c r="Y10" t="n">
-        <v>40</v>
+        <v>55.4</v>
       </c>
       <c r="Z10" t="n">
-        <v>28.6</v>
+        <v>27.6</v>
       </c>
       <c r="AA10" t="n">
-        <v>35</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:45</t>
+          <t>02:45</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Motherwell</t>
+          <t>Lokomotiv</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Aberdeen</t>
+          <t>Krylia Sovetov</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="E11" t="n">
-        <v>3.7</v>
+        <v>3.9</v>
       </c>
       <c r="F11" t="n">
         <v>4</v>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
       <c r="I11" t="n">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Scotland Premiership +</t>
+          <t>Russia Premier League</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⏭</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1422,74 +1448,74 @@
         </is>
       </c>
       <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
+      <c r="T11" t="n">
+        <v>53.9</v>
+      </c>
       <c r="U11" t="inlineStr"/>
       <c r="V11" t="n">
-        <v>46.6</v>
+        <v>50.1</v>
       </c>
       <c r="W11" t="n">
-        <v>28.8</v>
+        <v>31.3</v>
       </c>
       <c r="X11" t="n">
-        <v>24.7</v>
+        <v>18.6</v>
       </c>
       <c r="Y11" t="n">
-        <v>54.8</v>
+        <v>53.9</v>
       </c>
       <c r="Z11" t="n">
-        <v>34.2</v>
+        <v>34.1</v>
       </c>
       <c r="AA11" t="n">
-        <v>73</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Hapoel Beer Sheva</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Espanyol</t>
+          <t>Dinamo Zagreb</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2.2</v>
+        <v>3.7</v>
       </c>
       <c r="E12" t="n">
-        <v>3.4</v>
+        <v>3.8</v>
       </c>
       <c r="F12" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
+        <v>1.9</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
       <c r="I12" t="n">
-        <v>105</v>
+        <v>60</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Spain La Liga +</t>
+          <t>World UEFA Europa League</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>⏭</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M12" t="inlineStr"/>
@@ -1511,74 +1537,74 @@
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
+      <c r="T12" t="n">
+        <v>49.9</v>
+      </c>
       <c r="U12" t="inlineStr"/>
       <c r="V12" t="n">
-        <v>48.6</v>
+        <v>26</v>
       </c>
       <c r="W12" t="n">
-        <v>21</v>
+        <v>29.1</v>
       </c>
       <c r="X12" t="n">
+        <v>45</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="Z12" t="n">
         <v>30.5</v>
       </c>
-      <c r="Y12" t="n">
-        <v>55.2</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>29.5</v>
-      </c>
       <c r="AA12" t="n">
-        <v>105</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SV Meppen</t>
+          <t>AC Milan</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>FC Viktoria Köln</t>
+          <t>Benfica</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2.5</v>
+        <v>2.1</v>
       </c>
       <c r="E13" t="n">
         <v>3.7</v>
       </c>
       <c r="F13" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>무승부</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr"/>
+        <v>3.5</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
       <c r="I13" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Germany 3. Liga +</t>
+          <t>World UEFA Europa League</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>⏭</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>원정정배</t>
+          <t>홈정배</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -1600,69 +1626,69 @@
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
-      <c r="T13" t="inlineStr"/>
+      <c r="T13" t="n">
+        <v>50.2</v>
+      </c>
       <c r="U13" t="inlineStr"/>
       <c r="V13" t="n">
-        <v>20</v>
+        <v>46.4</v>
       </c>
       <c r="W13" t="n">
-        <v>40</v>
+        <v>25.6</v>
       </c>
       <c r="X13" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="Y13" t="n">
-        <v>60</v>
+        <v>50.2</v>
       </c>
       <c r="Z13" t="n">
-        <v>43.3</v>
+        <v>27.8</v>
       </c>
       <c r="AA13" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>03:00</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alaves</t>
+          <t>Atletico-MG</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Santos</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="E14" t="n">
-        <v>3.3</v>
+        <v>3.4</v>
       </c>
       <c r="F14" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>홈승</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
+        <v>4.3</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
       <c r="I14" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Spain La Liga +</t>
+          <t>World CONMEBOL Sudamericana</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>⚡</t>
+          <t>⏭</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1689,72 +1715,74 @@
         </is>
       </c>
       <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
+      <c r="T14" t="n">
+        <v>43.7</v>
+      </c>
       <c r="U14" t="inlineStr"/>
       <c r="V14" t="n">
-        <v>42.9</v>
+        <v>36.4</v>
       </c>
       <c r="W14" t="n">
-        <v>28.6</v>
+        <v>49.8</v>
       </c>
       <c r="X14" t="n">
-        <v>28.6</v>
+        <v>13.9</v>
       </c>
       <c r="Y14" t="n">
-        <v>61.9</v>
+        <v>43.7</v>
       </c>
       <c r="Z14" t="n">
-        <v>38.1</v>
+        <v>25.4</v>
       </c>
       <c r="AA14" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Londrina</t>
+          <t>Sturm Graz</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Ponte Preta</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>1.3</v>
+        <v>3.6</v>
       </c>
       <c r="E15" t="n">
-        <v>5.2</v>
+        <v>3.9</v>
       </c>
       <c r="F15" t="n">
-        <v>10.2</v>
+        <v>2</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Brazil Serie B +</t>
+          <t>World UEFA Europa League</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⏭</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1776,72 +1804,74 @@
         </is>
       </c>
       <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
+      <c r="T15" t="n">
+        <v>51.5</v>
+      </c>
       <c r="U15" t="inlineStr"/>
       <c r="V15" t="n">
-        <v>100</v>
+        <v>28.8</v>
       </c>
       <c r="W15" t="n">
-        <v>0</v>
+        <v>30.8</v>
       </c>
       <c r="X15" t="n">
-        <v>0</v>
+        <v>40.4</v>
       </c>
       <c r="Y15" t="n">
-        <v>100</v>
+        <v>51.5</v>
       </c>
       <c r="Z15" t="n">
-        <v>100</v>
+        <v>30.4</v>
       </c>
       <c r="AA15" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>03:00</t>
+          <t>02:45</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Ajax</t>
+          <t>Baltika</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Willem II</t>
+          <t>Zenit</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>1.1</v>
+        <v>4.2</v>
       </c>
       <c r="E16" t="n">
-        <v>9.199999999999999</v>
+        <v>3.5</v>
       </c>
       <c r="F16" t="n">
-        <v>17.2</v>
+        <v>1.9</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Netherlands Eredivisie +</t>
+          <t>Russia Premier League</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⏭</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>홈정배</t>
+          <t>원정정배</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -1863,57 +1893,69 @@
         </is>
       </c>
       <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
+      <c r="T16" t="n">
+        <v>57.5</v>
+      </c>
       <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
+      <c r="V16" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="W16" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="X16" t="n">
+        <v>36</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>30.7</v>
+      </c>
       <c r="AA16" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>03:45</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Stenhousemuir</t>
+          <t>Waldhof Mannheim</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Partick</t>
+          <t>Rot-Weiß Essen</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>2.8</v>
       </c>
       <c r="E17" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="F17" t="n">
-        <v>1.5</v>
+        <v>2.1</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="n">
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>7</v>
+        <v>60</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Scotland Championship +</t>
+          <t>Germany 3. Liga</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⏭</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1940,67 +1982,69 @@
         </is>
       </c>
       <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
+      <c r="T17" t="n">
+        <v>54.1</v>
+      </c>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="n">
-        <v>0</v>
+        <v>28.6</v>
       </c>
       <c r="W17" t="n">
-        <v>14.3</v>
+        <v>22.6</v>
       </c>
       <c r="X17" t="n">
-        <v>85.7</v>
+        <v>48.8</v>
       </c>
       <c r="Y17" t="n">
-        <v>57.1</v>
+        <v>54.1</v>
       </c>
       <c r="Z17" t="n">
-        <v>14.3</v>
+        <v>28.4</v>
       </c>
       <c r="AA17" t="n">
-        <v>7</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>01:45</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Elche</t>
+          <t>Omonia Nicosia</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Real Madrid</t>
+          <t>Celta Vigo</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>11.5</v>
+        <v>3.8</v>
       </c>
       <c r="E18" t="n">
-        <v>6.9</v>
+        <v>3.4</v>
       </c>
       <c r="F18" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="n">
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Spain La Liga +</t>
+          <t>World UEFA Europa League</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⏭</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2027,57 +2071,69 @@
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
+      <c r="T18" t="n">
+        <v>56.5</v>
+      </c>
       <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
+      <c r="V18" t="n">
+        <v>33.1</v>
+      </c>
+      <c r="W18" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="X18" t="n">
+        <v>40.4</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>56.5</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>32.6</v>
+      </c>
       <c r="AA18" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Vasco DA Gama</t>
+          <t>FC Ingolstadt 04</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Santa Fe</t>
+          <t>Hoffenheim II</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1.5</v>
+        <v>1.8</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="F19" t="n">
-        <v>7.2</v>
+        <v>3.3</v>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>2</v>
+        <v>60</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>World CONMEBOL Sudamericana +</t>
+          <t>Germany 3. Liga</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>❓</t>
+          <t>⏭</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -2104,25 +2160,838 @@
         </is>
       </c>
       <c r="S19" t="inlineStr"/>
-      <c r="T19" t="inlineStr"/>
+      <c r="T19" t="n">
+        <v>55.4</v>
+      </c>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="n">
-        <v>100</v>
+        <v>36.5</v>
       </c>
       <c r="W19" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="X19" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Preußen Münster</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>FC Saarbrücken</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="E20" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
         <v>0</v>
       </c>
-      <c r="X19" t="n">
+      <c r="I20" t="n">
+        <v>60</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Germany 3. Liga</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="n">
+        <v>54</v>
+      </c>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="W20" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="X20" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>54</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="AA20" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Anderlecht</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="n">
         <v>0</v>
       </c>
-      <c r="Y19" t="n">
-        <v>50</v>
-      </c>
-      <c r="Z19" t="n">
-        <v>50</v>
-      </c>
-      <c r="AA19" t="n">
+      <c r="I21" t="n">
+        <v>60</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>World UEFA Europa League</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="W21" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="X21" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Fortuna Köln</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>SV Wehen</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>60</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Germany 3. Liga</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="n">
+        <v>54</v>
+      </c>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="W22" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="X22" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>54</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Once Caldas</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Deportes Tolima</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
         <v>2</v>
+      </c>
+      <c r="E23" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>48</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Colombia Primera A</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="W23" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="X23" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>42.1</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Levante</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Athletic Club</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>60</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Spain La Liga</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="W24" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="X24" t="n">
+        <v>34</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>52.6</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>LDU de Quito</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Palmeiras</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>24</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>World CONMEBOL Libertadores</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="W25" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="X25" t="n">
+        <v>47</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>49.7</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Deportivo La Coruna</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>60</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Spain La Liga</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="W26" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="X26" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>FK Yenisey</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Arsenal Tula</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>3</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>60</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Russia First League</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>홈정배</t>
+        </is>
+      </c>
+      <c r="M27" t="n">
+        <v>33</v>
+      </c>
+      <c r="N27" t="n">
+        <v>42</v>
+      </c>
+      <c r="O27" t="n">
+        <v>25</v>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S27" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="T27" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="U27" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="V27" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="W27" t="n">
+        <v>30</v>
+      </c>
+      <c r="X27" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>53.8</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>00:30</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Rodina Moskva</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Rubin</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>60</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Russia Premier League</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>⏭</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>원정정배</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="n">
+        <v>36</v>
+      </c>
+      <c r="W28" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="X28" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>33</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>